<commit_message>
Exclusion des agents à 0 tenue : liste 1 à 6 tenues + synthèse mises à jour
</commit_message>
<xml_diff>
--- a/Synthese_par_service_Saint-Louis.xlsx
+++ b/Synthese_par_service_Saint-Louis.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Synthèse par service" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthèse par service'!$A$1:$F$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Synthèse par service'!$A$1:$E$59</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,15 +455,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F64"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,12 +473,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Nb agents</t>
+          <t>Nb agents (hors 0 tenue)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Agents &lt; 7 tenues</t>
+          <t>Agents 1 à 6 tenues</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -488,11 +487,6 @@
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Dont 0 tenue (incomplet)</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Tenues moy. / agent</t>
         </is>
@@ -505,19 +499,16 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>163</v>
+        <v>143</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.9570552147239264</v>
+        <v>0.951048951048951</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>4.7</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="3">
@@ -527,19 +518,16 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>0.9375</v>
+        <v>0.9310344827586207</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="4">
@@ -549,41 +537,35 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>81</v>
+        <v>56</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0.9876543209876543</v>
+        <v>0.9821428571428571</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>4.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BLOC OBSTETRIQUE</t>
+          <t>IMAGERIE A</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.9824561403508771</v>
+        <v>0.9795918367346939</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>1.8</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="6">
@@ -593,63 +575,54 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.864406779661017</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>5.1</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>IMAGERIE A</t>
+          <t>MIMIR</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>0.9807692307692307</v>
+        <v>0.9777777777777777</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>4.8</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>MIMIR</t>
+          <t>MED B/NEURO</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0.9791666666666666</v>
+        <v>0.8913043478260869</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>5.1</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="9">
@@ -659,85 +632,73 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0.9791666666666666</v>
+        <v>0.975</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>4.7</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>MED B/NEURO</t>
+          <t>POOL REMPL</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.9</v>
+        <v>0.926829268292683</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ONCOLOGIE HC</t>
+          <t>MED POLY 3N</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0.9772727272727273</v>
+        <v>0.9487179487179487</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>4.1</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>POOL REMPL</t>
+          <t>PHARMACIE</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0.9333333333333333</v>
+        <v>1</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>5.4</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="13">
@@ -747,19 +708,16 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.7358490566037735</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="14">
@@ -769,239 +727,206 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9210526315789473</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>4.7</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>MED POLY 3N</t>
+          <t>CHIR C1/VISCERALE</t>
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.9512195121951219</v>
+        <v>1</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" s="2" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PHARMACIE</t>
+          <t>ONCOLOGIE HC</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1</v>
+        <v>0.9714285714285714</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>3.1</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>CENTRE 15</t>
+          <t>PNEUMO</t>
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>1</v>
+        <v>0.8918918918918919</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>0.2</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>CHIR C1/VISCERALE</t>
+          <t>ONCOLOGIE HDJ</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PNEUMO</t>
+          <t>DIABETO/NEPHRO</t>
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>0.9024390243902439</v>
+        <v>0.9375</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F19" s="2" t="n">
-        <v>5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>CHIR ORTHO</t>
+          <t>KINESI</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>0.8974358974358975</v>
+        <v>0.9666666666666667</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="F20" s="2" t="n">
-        <v>4.4</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ONCOLOGIE HDJ</t>
+          <t>CHIR E/VASCULAIRE/URO</t>
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="2" t="n">
-        <v>5.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>DIABETO/NEPHRO</t>
+          <t>CHIR ORTHO</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="E22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F22" s="2" t="n">
-        <v>5.1</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CHIR E/VASCULAIRE/URO</t>
+          <t>GYNECOLOGIE</t>
         </is>
       </c>
       <c r="B23" s="2" t="n">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>0.9117647058823529</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="E23" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F23" s="2" t="n">
-        <v>5.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>KINESI</t>
+          <t>MED E/GASTRO ENTERO</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>0.9666666666666667</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="2" t="n">
-        <v>5.9</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="25">
@@ -1011,41 +936,35 @@
         </is>
       </c>
       <c r="B25" s="2" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>0.9655172413793104</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F25" s="2" t="n">
-        <v>4</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GYNECOLOGIE</t>
+          <t>BLOC OP</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.9310344827586207</v>
+        <v>0.7826086956521739</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>5.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
@@ -1055,591 +974,510 @@
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>0.9615384615384616</v>
+        <v>0.9473684210526315</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>LABORATOIRES</t>
+          <t>OBSTETRIQUE</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>1</v>
+        <v>0.9473684210526315</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>1.2</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>MED E/GASTRO ENTERO</t>
+          <t>BLOC OBSTETRIQUE</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.96</v>
+        <v>0.9444444444444444</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F29" s="2" t="n">
-        <v>4.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>MED AIGUE GERIATRIQUE</t>
+          <t>I.F.S.I</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>0.6216216216216216</v>
+        <v>1</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>3.8</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>I.F.S.I</t>
+          <t>CMPE</t>
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>2.2</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>BLOC OP</t>
+          <t>MED AIGUE GERIATRIQUE</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>0.8</v>
+        <v>0.4814814814814815</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>4.6</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>OBSTETRIQUE</t>
+          <t>ANAPATH ( LABO C )</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>0.9473684210526315</v>
+        <v>1</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="2" t="n">
-        <v>5.9</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>S.M.U.R</t>
+          <t>CE ORL</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>1</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>1.9</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>CE ORL</t>
+          <t>CELLULE D' ORDONNANCEMENT</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>0.875</v>
+        <v>1</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F35" s="2" t="n">
-        <v>4.2</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>CMPE</t>
+          <t>CARDIO H. SEMAINE</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C36" s="2" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1</v>
+        <v>0.5263157894736842</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>4.1</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>CARDIO H. COMPLETE</t>
+          <t>CO GYNECO</t>
         </is>
       </c>
       <c r="B37" s="2" t="n">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C37" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0.4814814814814815</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="F37" s="2" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>CO GYNECO</t>
+          <t>CHIR AMBUL</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C38" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0.7222222222222222</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>4.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>CHIR AMBUL</t>
+          <t>ENDOSCOPIE DIGESTIVE</t>
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C39" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F39" s="2" t="n">
-        <v>4.6</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ENDOSCOPIE DIGESTIVE</t>
+          <t>CE CHIR</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C40" s="2" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>3.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ANAPATH ( LABO C )</t>
+          <t>E C G</t>
         </is>
       </c>
       <c r="B41" s="2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C41" s="2" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>1</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" s="2" t="n">
-        <v>4.2</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>BRANCARD</t>
+          <t>E E G</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="C42" s="2" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>3.9</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>CE OPHTAL</t>
+          <t>LABORATOIRES</t>
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C43" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D43" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F43" s="2" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>CELLULE D' ORDONNANCEMENT</t>
+          <t>CE OPHTAL</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D44" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="2" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>CARDIO H. SEMAINE</t>
+          <t>CARDIO H. COMPLETE</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>0.55</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F45" s="2" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>E C G</t>
+          <t>S.M.U.R</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>0.6875</v>
+        <v>1</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F46" s="2" t="n">
-        <v>4.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>CE CHIR</t>
+          <t>C.E.CHIR A .URO</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>E E G</t>
+          <t>U.M.D.S.P</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C48" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" s="2" t="n">
-        <v>5.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>HDJ MEDECINE</t>
+          <t>CE STOMATO (TENUES)</t>
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C49" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F49" s="2" t="n">
-        <v>3.6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>U.M.D.S.P</t>
+          <t>HDJ MEDECINE</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="2" t="n">
-        <v>2.5</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>C.E.CHIR A .URO</t>
+          <t>MED PREV</t>
         </is>
       </c>
       <c r="B51" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>0.8333333333333334</v>
+        <v>1</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F51" s="2" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>CE STOMATO (TENUES)</t>
+          <t>BRANCARD</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="2" t="n">
-        <v>4.2</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>U.C.S.A</t>
+          <t>CENTRE 15</t>
         </is>
       </c>
       <c r="B53" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D53" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="F53" s="2" t="n">
-        <v>0.4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="54">
@@ -1649,32 +1487,29 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D54" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="F54" s="2" t="n">
-        <v>2.2</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>AMPHITH</t>
+          <t>CE STOMATO</t>
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C55" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D55" s="3" t="n">
         <v>1</v>
@@ -1682,208 +1517,102 @@
       <c r="E55" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F55" s="2" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>MED PREV</t>
+          <t>CE LABO</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D56" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F56" s="2" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>U.R.C</t>
+          <t>U.C.S.A  CITADELLE</t>
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D57" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="F57" s="2" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>U.C.S.A  CITADELLE</t>
+          <t>U.C.S.A</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="2" t="n">
         <v>2</v>
-      </c>
-      <c r="D58" s="3" t="n">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="E58" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F58" s="2" t="n">
-        <v>6.3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>CE STOMATO</t>
+          <t>U.C.S.A  CASERNE</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D59" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F59" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>CE LABO</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D60" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F60" s="2" t="n">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>D.I.M.</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C61" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>U.C.S.A  CASERNE</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F62" s="2" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>BLOC GYNECO</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F63" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>TOTAL GÉNÉRAL</t>
         </is>
       </c>
-      <c r="B64" s="4" t="n">
-        <v>1735</v>
-      </c>
-      <c r="C64" s="4" t="n">
-        <v>1586</v>
-      </c>
-      <c r="D64" s="5" t="n">
-        <v>0.914121037463977</v>
-      </c>
-      <c r="E64" s="4" t="n">
-        <v>323</v>
-      </c>
-      <c r="F64" s="4" t="inlineStr"/>
+      <c r="B60" s="4" t="n">
+        <v>1412</v>
+      </c>
+      <c r="C60" s="4" t="n">
+        <v>1263</v>
+      </c>
+      <c r="D60" s="5" t="n">
+        <v>0.8944759206798867</v>
+      </c>
+      <c r="E60" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F63"/>
+  <autoFilter ref="A1:E59"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>